<commit_message>
Deploy: silver ore + full re-extract in trade figures; refreshed workbooks
🤖 Generated with [Claude Code](https://claude.com/claude-code)
</commit_message>
<xml_diff>
--- a/projects/NZIPL/docs/trade_data/latest_2024/NZIPL_2024_CountryTotals_Balance_USDmn.xlsx
+++ b/projects/NZIPL/docs/trade_data/latest_2024/NZIPL_2024_CountryTotals_Balance_USDmn.xlsx
@@ -94,7 +94,7 @@
     <t xml:space="preserve">Generated</t>
   </si>
   <si>
-    <t xml:space="preserve">2026-07-10</t>
+    <t xml:space="preserve">2026-07-11</t>
   </si>
   <si>
     <t xml:space="preserve">ISO3</t>
@@ -1560,7 +1560,7 @@
         <v>28</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>-22022.551</v>
+        <v>-20850.869</v>
       </c>
     </row>
     <row r="3">
@@ -1571,7 +1571,7 @@
         <v>34</v>
       </c>
       <c r="C3" s="2" t="n">
-        <v>-28633.735</v>
+        <v>-28777.208</v>
       </c>
     </row>
     <row r="4">
@@ -1582,7 +1582,7 @@
         <v>32</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>14842.918</v>
+        <v>15661.444</v>
       </c>
     </row>
     <row r="5">
@@ -1593,7 +1593,7 @@
         <v>36</v>
       </c>
       <c r="C5" s="2" t="n">
-        <v>-1931.376</v>
+        <v>-2119.954</v>
       </c>
     </row>
     <row r="6">
@@ -1604,7 +1604,7 @@
         <v>44</v>
       </c>
       <c r="C6" s="2" t="n">
-        <v>8850.536</v>
+        <v>8789.411</v>
       </c>
     </row>
     <row r="7">
@@ -1615,7 +1615,7 @@
         <v>46</v>
       </c>
       <c r="C7" s="2" t="n">
-        <v>-5110.724</v>
+        <v>-5150.993</v>
       </c>
     </row>
     <row r="8">
@@ -1626,7 +1626,7 @@
         <v>38</v>
       </c>
       <c r="C8" s="2" t="n">
-        <v>-37.889</v>
+        <v>-73.697</v>
       </c>
     </row>
     <row r="9">
@@ -1637,7 +1637,7 @@
         <v>42</v>
       </c>
       <c r="C9" s="2" t="n">
-        <v>-399.981</v>
+        <v>-461.276</v>
       </c>
     </row>
     <row r="10">
@@ -1648,7 +1648,7 @@
         <v>60</v>
       </c>
       <c r="C10" s="2" t="n">
-        <v>-4889.978</v>
+        <v>-4879.482</v>
       </c>
     </row>
     <row r="11">
@@ -1659,7 +1659,7 @@
         <v>48</v>
       </c>
       <c r="C11" s="2" t="n">
-        <v>-5157.201</v>
+        <v>-5456.341</v>
       </c>
     </row>
     <row r="12">
@@ -1670,7 +1670,7 @@
         <v>50</v>
       </c>
       <c r="C12" s="2" t="n">
-        <v>-3511.341</v>
+        <v>-3509.52</v>
       </c>
     </row>
     <row r="13">
@@ -1681,7 +1681,7 @@
         <v>64</v>
       </c>
       <c r="C13" s="2" t="n">
-        <v>-1814.262</v>
+        <v>-1681.247</v>
       </c>
     </row>
     <row r="14">
@@ -1692,7 +1692,7 @@
         <v>58</v>
       </c>
       <c r="C14" s="2" t="n">
-        <v>-1872.794</v>
+        <v>-1887.065</v>
       </c>
     </row>
     <row r="15">
@@ -1703,7 +1703,7 @@
         <v>30</v>
       </c>
       <c r="C15" s="2" t="n">
-        <v>12515.477</v>
+        <v>12449.536</v>
       </c>
     </row>
     <row r="16">
@@ -1714,7 +1714,7 @@
         <v>54</v>
       </c>
       <c r="C16" s="2" t="n">
-        <v>-4748.775</v>
+        <v>-4552.059</v>
       </c>
     </row>
     <row r="17">
@@ -1725,7 +1725,7 @@
         <v>56</v>
       </c>
       <c r="C17" s="2" t="n">
-        <v>996.034</v>
+        <v>818.959</v>
       </c>
     </row>
     <row r="18">
@@ -1736,7 +1736,7 @@
         <v>52</v>
       </c>
       <c r="C18" s="2" t="n">
-        <v>30433.466</v>
+        <v>30262.463</v>
       </c>
     </row>
     <row r="19">
@@ -1747,7 +1747,7 @@
         <v>66</v>
       </c>
       <c r="C19" s="2" t="n">
-        <v>717.13</v>
+        <v>717.029</v>
       </c>
     </row>
     <row r="20">
@@ -1758,7 +1758,7 @@
         <v>74</v>
       </c>
       <c r="C20" s="2" t="n">
-        <v>-1467.928</v>
+        <v>-1509.888</v>
       </c>
     </row>
     <row r="21">
@@ -1769,7 +1769,7 @@
         <v>40</v>
       </c>
       <c r="C21" s="2" t="n">
-        <v>1706.106</v>
+        <v>1512.844</v>
       </c>
     </row>
     <row r="22">
@@ -1780,7 +1780,7 @@
         <v>88</v>
       </c>
       <c r="C22" s="2" t="n">
-        <v>-3865.699</v>
+        <v>-3866.421</v>
       </c>
     </row>
     <row r="23">
@@ -1791,29 +1791,29 @@
         <v>84</v>
       </c>
       <c r="C23" s="2" t="n">
-        <v>88.046</v>
+        <v>80.384</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="s">
-        <v>75</v>
+        <v>81</v>
       </c>
       <c r="B24" t="s">
-        <v>76</v>
+        <v>82</v>
       </c>
       <c r="C24" s="2" t="n">
-        <v>-3899.87</v>
+        <v>-437.809</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="s">
-        <v>81</v>
+        <v>75</v>
       </c>
       <c r="B25" t="s">
-        <v>82</v>
+        <v>76</v>
       </c>
       <c r="C25" s="2" t="n">
-        <v>-371.956</v>
+        <v>-3899.247</v>
       </c>
     </row>
     <row r="26">
@@ -1824,7 +1824,7 @@
         <v>86</v>
       </c>
       <c r="C26" s="2" t="n">
-        <v>-3584.224</v>
+        <v>-3841.963</v>
       </c>
     </row>
     <row r="27">
@@ -1835,7 +1835,7 @@
         <v>92</v>
       </c>
       <c r="C27" s="2" t="n">
-        <v>-391.767</v>
+        <v>-391.824</v>
       </c>
     </row>
     <row r="28">
@@ -1857,7 +1857,7 @@
         <v>70</v>
       </c>
       <c r="C29" s="2" t="n">
-        <v>115.549</v>
+        <v>115.492</v>
       </c>
     </row>
     <row r="30">
@@ -1868,7 +1868,7 @@
         <v>80</v>
       </c>
       <c r="C30" s="2" t="n">
-        <v>-4774.137</v>
+        <v>-4774.211</v>
       </c>
     </row>
     <row r="31">
@@ -1879,7 +1879,7 @@
         <v>78</v>
       </c>
       <c r="C31" s="2" t="n">
-        <v>565.244</v>
+        <v>565.041</v>
       </c>
     </row>
   </sheetData>
@@ -1917,7 +1917,7 @@
         <v>28</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>-150644.262</v>
+        <v>-150269.795</v>
       </c>
     </row>
     <row r="3">
@@ -1928,7 +1928,7 @@
         <v>30</v>
       </c>
       <c r="C3" s="2" t="n">
-        <v>97481.889</v>
+        <v>97477.024</v>
       </c>
     </row>
     <row r="4">
@@ -1939,7 +1939,7 @@
         <v>32</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>1653.715</v>
+        <v>1647.508</v>
       </c>
     </row>
     <row r="5">
@@ -1950,7 +1950,7 @@
         <v>34</v>
       </c>
       <c r="C5" s="2" t="n">
-        <v>-11249.045</v>
+        <v>-11253.088</v>
       </c>
     </row>
     <row r="6">
@@ -1961,7 +1961,7 @@
         <v>36</v>
       </c>
       <c r="C6" s="2" t="n">
-        <v>-14859.898</v>
+        <v>-14807.647</v>
       </c>
     </row>
     <row r="7">
@@ -1972,7 +1972,7 @@
         <v>38</v>
       </c>
       <c r="C7" s="2" t="n">
-        <v>-4762.183</v>
+        <v>-4764.029</v>
       </c>
     </row>
     <row r="8">
@@ -1983,7 +1983,7 @@
         <v>40</v>
       </c>
       <c r="C8" s="2" t="n">
-        <v>36326.001</v>
+        <v>36320.872</v>
       </c>
     </row>
     <row r="9">
@@ -1994,7 +1994,7 @@
         <v>42</v>
       </c>
       <c r="C9" s="2" t="n">
-        <v>5925.397</v>
+        <v>5907.096</v>
       </c>
     </row>
     <row r="10">
@@ -2005,7 +2005,7 @@
         <v>44</v>
       </c>
       <c r="C10" s="2" t="n">
-        <v>2356.2</v>
+        <v>2351.431</v>
       </c>
     </row>
     <row r="11">
@@ -2016,7 +2016,7 @@
         <v>46</v>
       </c>
       <c r="C11" s="2" t="n">
-        <v>-3918.67</v>
+        <v>-3910.373</v>
       </c>
     </row>
     <row r="12">
@@ -2027,7 +2027,7 @@
         <v>48</v>
       </c>
       <c r="C12" s="2" t="n">
-        <v>-2122.637</v>
+        <v>-2121.906</v>
       </c>
     </row>
     <row r="13">
@@ -2038,7 +2038,7 @@
         <v>50</v>
       </c>
       <c r="C13" s="2" t="n">
-        <v>-3170.678</v>
+        <v>-3168.155</v>
       </c>
     </row>
     <row r="14">
@@ -2049,7 +2049,7 @@
         <v>52</v>
       </c>
       <c r="C14" s="2" t="n">
-        <v>34823.702</v>
+        <v>34579.554</v>
       </c>
     </row>
     <row r="15">
@@ -2060,7 +2060,7 @@
         <v>54</v>
       </c>
       <c r="C15" s="2" t="n">
-        <v>-10217.752</v>
+        <v>-10217.556</v>
       </c>
     </row>
     <row r="16">
@@ -2071,7 +2071,7 @@
         <v>56</v>
       </c>
       <c r="C16" s="2" t="n">
-        <v>-2898.603</v>
+        <v>-2904.807</v>
       </c>
     </row>
     <row r="17">
@@ -2082,7 +2082,7 @@
         <v>58</v>
       </c>
       <c r="C17" s="2" t="n">
-        <v>-2821.401</v>
+        <v>-2820.374</v>
       </c>
     </row>
     <row r="18">
@@ -2093,7 +2093,7 @@
         <v>60</v>
       </c>
       <c r="C18" s="2" t="n">
-        <v>-8062.555</v>
+        <v>-8069.998</v>
       </c>
     </row>
     <row r="19">
@@ -2104,7 +2104,7 @@
         <v>62</v>
       </c>
       <c r="C19" s="2" t="n">
-        <v>11532.467</v>
+        <v>11540.177</v>
       </c>
     </row>
     <row r="20">
@@ -2115,7 +2115,7 @@
         <v>64</v>
       </c>
       <c r="C20" s="2" t="n">
-        <v>-3355.393</v>
+        <v>-3361.712</v>
       </c>
     </row>
     <row r="21">
@@ -2126,7 +2126,7 @@
         <v>66</v>
       </c>
       <c r="C21" s="2" t="n">
-        <v>-1122.082</v>
+        <v>-1119.994</v>
       </c>
     </row>
     <row r="22">
@@ -2137,7 +2137,7 @@
         <v>68</v>
       </c>
       <c r="C22" s="2" t="n">
-        <v>8249.352</v>
+        <v>8248.044</v>
       </c>
     </row>
     <row r="23">
@@ -2148,7 +2148,7 @@
         <v>70</v>
       </c>
       <c r="C23" s="2" t="n">
-        <v>-183.338</v>
+        <v>-195.65</v>
       </c>
     </row>
     <row r="24">
@@ -2159,7 +2159,7 @@
         <v>72</v>
       </c>
       <c r="C24" s="2" t="n">
-        <v>21567.723</v>
+        <v>21565.985</v>
       </c>
     </row>
     <row r="25">
@@ -2170,7 +2170,7 @@
         <v>74</v>
       </c>
       <c r="C25" s="2" t="n">
-        <v>-68.942</v>
+        <v>-68.018</v>
       </c>
     </row>
     <row r="26">
@@ -2181,7 +2181,7 @@
         <v>76</v>
       </c>
       <c r="C26" s="2" t="n">
-        <v>-339.788</v>
+        <v>-342.557</v>
       </c>
     </row>
     <row r="27">
@@ -2192,7 +2192,7 @@
         <v>78</v>
       </c>
       <c r="C27" s="2" t="n">
-        <v>1110.3</v>
+        <v>1121.952</v>
       </c>
     </row>
     <row r="28">
@@ -2203,7 +2203,7 @@
         <v>80</v>
       </c>
       <c r="C28" s="2" t="n">
-        <v>-2841.619</v>
+        <v>-2843.301</v>
       </c>
     </row>
     <row r="29">
@@ -2214,7 +2214,7 @@
         <v>82</v>
       </c>
       <c r="C29" s="2" t="n">
-        <v>893.986</v>
+        <v>890.16</v>
       </c>
     </row>
     <row r="30">
@@ -2225,7 +2225,7 @@
         <v>84</v>
       </c>
       <c r="C30" s="2" t="n">
-        <v>218.894</v>
+        <v>219.529</v>
       </c>
     </row>
     <row r="31">
@@ -2236,7 +2236,7 @@
         <v>86</v>
       </c>
       <c r="C31" s="2" t="n">
-        <v>-3858.263</v>
+        <v>-3856.223</v>
       </c>
     </row>
   </sheetData>
@@ -2274,7 +2274,7 @@
         <v>34</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>582.828</v>
+        <v>127.331</v>
       </c>
     </row>
     <row r="3">
@@ -2285,7 +2285,7 @@
         <v>32</v>
       </c>
       <c r="C3" s="2" t="n">
-        <v>3003.438</v>
+        <v>3815.04</v>
       </c>
     </row>
     <row r="4">
@@ -2296,7 +2296,7 @@
         <v>28</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>-10172.04</v>
+        <v>-9508.971</v>
       </c>
     </row>
     <row r="5">
@@ -2307,7 +2307,7 @@
         <v>36</v>
       </c>
       <c r="C5" s="2" t="n">
-        <v>-3342.258</v>
+        <v>-3337.162</v>
       </c>
     </row>
     <row r="6">
@@ -2318,7 +2318,7 @@
         <v>48</v>
       </c>
       <c r="C6" s="2" t="n">
-        <v>-504.186</v>
+        <v>-758.947</v>
       </c>
     </row>
     <row r="7">
@@ -2329,7 +2329,7 @@
         <v>50</v>
       </c>
       <c r="C7" s="2" t="n">
-        <v>-38.434</v>
+        <v>-696.892</v>
       </c>
     </row>
     <row r="8">
@@ -2340,7 +2340,7 @@
         <v>44</v>
       </c>
       <c r="C8" s="2" t="n">
-        <v>2304.096</v>
+        <v>2130.688</v>
       </c>
     </row>
     <row r="9">
@@ -2351,7 +2351,7 @@
         <v>38</v>
       </c>
       <c r="C9" s="2" t="n">
-        <v>-85.273</v>
+        <v>1.611</v>
       </c>
     </row>
     <row r="10">
@@ -2362,29 +2362,29 @@
         <v>46</v>
       </c>
       <c r="C10" s="2" t="n">
-        <v>-413.769</v>
+        <v>-1408.683</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>67</v>
+        <v>57</v>
       </c>
       <c r="B11" t="s">
-        <v>68</v>
+        <v>58</v>
       </c>
       <c r="C11" s="2" t="n">
-        <v>9776.654</v>
+        <v>384.929</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>57</v>
+        <v>67</v>
       </c>
       <c r="B12" t="s">
-        <v>58</v>
+        <v>68</v>
       </c>
       <c r="C12" s="2" t="n">
-        <v>-115.551</v>
+        <v>9776.71</v>
       </c>
     </row>
     <row r="13">
@@ -2395,7 +2395,7 @@
         <v>42</v>
       </c>
       <c r="C13" s="2" t="n">
-        <v>-6422.175</v>
+        <v>-6534.434</v>
       </c>
     </row>
     <row r="14">
@@ -2428,7 +2428,7 @@
         <v>64</v>
       </c>
       <c r="C16" s="2" t="n">
-        <v>-357.146</v>
+        <v>156.159</v>
       </c>
     </row>
     <row r="17">
@@ -2439,7 +2439,7 @@
         <v>78</v>
       </c>
       <c r="C17" s="2" t="n">
-        <v>-1744.981</v>
+        <v>-1839.357</v>
       </c>
     </row>
     <row r="18">
@@ -2450,7 +2450,7 @@
         <v>60</v>
       </c>
       <c r="C18" s="2" t="n">
-        <v>-2258.176</v>
+        <v>-2258.297</v>
       </c>
     </row>
     <row r="19">
@@ -2461,7 +2461,7 @@
         <v>40</v>
       </c>
       <c r="C19" s="2" t="n">
-        <v>1538.752</v>
+        <v>1591.753</v>
       </c>
     </row>
     <row r="20">
@@ -2472,7 +2472,7 @@
         <v>54</v>
       </c>
       <c r="C20" s="2" t="n">
-        <v>-4446.444</v>
+        <v>-4446.379</v>
       </c>
     </row>
     <row r="21">
@@ -2483,7 +2483,7 @@
         <v>62</v>
       </c>
       <c r="C21" s="2" t="n">
-        <v>542.53</v>
+        <v>660.044</v>
       </c>
     </row>
     <row r="22">
@@ -2494,7 +2494,7 @@
         <v>70</v>
       </c>
       <c r="C22" s="2" t="n">
-        <v>493.875</v>
+        <v>878.291</v>
       </c>
     </row>
     <row r="23">
@@ -2505,29 +2505,29 @@
         <v>56</v>
       </c>
       <c r="C23" s="2" t="n">
-        <v>-1701.245</v>
+        <v>-1635.953</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="s">
-        <v>87</v>
+        <v>73</v>
       </c>
       <c r="B24" t="s">
-        <v>88</v>
+        <v>74</v>
       </c>
       <c r="C24" s="2" t="n">
-        <v>609.415</v>
+        <v>626.521</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="s">
-        <v>73</v>
+        <v>87</v>
       </c>
       <c r="B25" t="s">
-        <v>74</v>
+        <v>88</v>
       </c>
       <c r="C25" s="2" t="n">
-        <v>686.788</v>
+        <v>636.895</v>
       </c>
     </row>
     <row r="26">
@@ -2549,7 +2549,7 @@
         <v>92</v>
       </c>
       <c r="C27" s="2" t="n">
-        <v>-432.215</v>
+        <v>-451.248</v>
       </c>
     </row>
     <row r="28">
@@ -2560,7 +2560,7 @@
         <v>82</v>
       </c>
       <c r="C28" s="2" t="n">
-        <v>-43.456</v>
+        <v>-252.842</v>
       </c>
     </row>
     <row r="29">
@@ -2571,7 +2571,7 @@
         <v>94</v>
       </c>
       <c r="C29" s="2" t="n">
-        <v>-1180.497</v>
+        <v>-1172.327</v>
       </c>
     </row>
     <row r="30">
@@ -2582,7 +2582,7 @@
         <v>76</v>
       </c>
       <c r="C30" s="2" t="n">
-        <v>-1258.678</v>
+        <v>-1355.359</v>
       </c>
     </row>
     <row r="31">
@@ -2593,7 +2593,7 @@
         <v>80</v>
       </c>
       <c r="C31" s="2" t="n">
-        <v>-1561.049</v>
+        <v>-1566.448</v>
       </c>
     </row>
   </sheetData>
@@ -2631,7 +2631,7 @@
         <v>28</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>-107173.038</v>
+        <v>-110113.585</v>
       </c>
     </row>
     <row r="3">
@@ -2642,7 +2642,7 @@
         <v>34</v>
       </c>
       <c r="C3" s="2" t="n">
-        <v>-51728.599</v>
+        <v>-51680.918</v>
       </c>
     </row>
     <row r="4">
@@ -2653,7 +2653,7 @@
         <v>32</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>34890.123</v>
+        <v>34846.254</v>
       </c>
     </row>
     <row r="5">
@@ -2664,7 +2664,7 @@
         <v>36</v>
       </c>
       <c r="C5" s="2" t="n">
-        <v>-1631.684</v>
+        <v>-1823.285</v>
       </c>
     </row>
     <row r="6">
@@ -2675,7 +2675,7 @@
         <v>30</v>
       </c>
       <c r="C6" s="2" t="n">
-        <v>96127.242</v>
+        <v>96153.786</v>
       </c>
     </row>
     <row r="7">
@@ -2686,7 +2686,7 @@
         <v>42</v>
       </c>
       <c r="C7" s="2" t="n">
-        <v>-1643.539</v>
+        <v>-1584.566</v>
       </c>
     </row>
     <row r="8">
@@ -2708,7 +2708,7 @@
         <v>38</v>
       </c>
       <c r="C9" s="2" t="n">
-        <v>-2072.442</v>
+        <v>-2442.947</v>
       </c>
     </row>
     <row r="10">
@@ -2719,7 +2719,7 @@
         <v>60</v>
       </c>
       <c r="C10" s="2" t="n">
-        <v>13951.002</v>
+        <v>14152.773</v>
       </c>
     </row>
     <row r="11">
@@ -2730,7 +2730,7 @@
         <v>40</v>
       </c>
       <c r="C11" s="2" t="n">
-        <v>33482.708</v>
+        <v>33510.863</v>
       </c>
     </row>
     <row r="12">
@@ -2752,7 +2752,7 @@
         <v>44</v>
       </c>
       <c r="C13" s="2" t="n">
-        <v>1030.009</v>
+        <v>1030.479</v>
       </c>
     </row>
     <row r="14">
@@ -2763,7 +2763,7 @@
         <v>64</v>
       </c>
       <c r="C14" s="2" t="n">
-        <v>-4343.901</v>
+        <v>-4331.454</v>
       </c>
     </row>
     <row r="15">
@@ -2774,7 +2774,7 @@
         <v>50</v>
       </c>
       <c r="C15" s="2" t="n">
-        <v>-9853.328</v>
+        <v>-9853.48</v>
       </c>
     </row>
     <row r="16">
@@ -2796,7 +2796,7 @@
         <v>58</v>
       </c>
       <c r="C17" s="2" t="n">
-        <v>-8985.407</v>
+        <v>-9122.002</v>
       </c>
     </row>
     <row r="18">
@@ -2829,7 +2829,7 @@
         <v>66</v>
       </c>
       <c r="C20" s="2" t="n">
-        <v>-788.576</v>
+        <v>-462.741</v>
       </c>
     </row>
     <row r="21">
@@ -2851,7 +2851,7 @@
         <v>82</v>
       </c>
       <c r="C22" s="2" t="n">
-        <v>-3965.965</v>
+        <v>-3961.278</v>
       </c>
     </row>
     <row r="23">
@@ -2862,7 +2862,7 @@
         <v>86</v>
       </c>
       <c r="C23" s="2" t="n">
-        <v>-11099.553</v>
+        <v>-11063.222</v>
       </c>
     </row>
     <row r="24">
@@ -2873,7 +2873,7 @@
         <v>52</v>
       </c>
       <c r="C24" s="2" t="n">
-        <v>31712.554</v>
+        <v>31682.968</v>
       </c>
     </row>
     <row r="25">
@@ -2884,7 +2884,7 @@
         <v>88</v>
       </c>
       <c r="C25" s="2" t="n">
-        <v>4730.495</v>
+        <v>4730.252</v>
       </c>
     </row>
     <row r="26">
@@ -2906,7 +2906,7 @@
         <v>62</v>
       </c>
       <c r="C27" s="2" t="n">
-        <v>6093.44</v>
+        <v>6093.325</v>
       </c>
     </row>
     <row r="28">
@@ -2917,7 +2917,7 @@
         <v>70</v>
       </c>
       <c r="C28" s="2" t="n">
-        <v>-5845.13</v>
+        <v>-5795.857</v>
       </c>
     </row>
     <row r="29">
@@ -2939,7 +2939,7 @@
         <v>68</v>
       </c>
       <c r="C30" s="2" t="n">
-        <v>8723.084</v>
+        <v>8720.494</v>
       </c>
     </row>
     <row r="31">
@@ -2950,7 +2950,7 @@
         <v>76</v>
       </c>
       <c r="C31" s="2" t="n">
-        <v>-2175.469</v>
+        <v>-2176.541</v>
       </c>
     </row>
   </sheetData>
@@ -2988,7 +2988,7 @@
         <v>28</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>21329.163</v>
+        <v>21534.259</v>
       </c>
     </row>
     <row r="3">
@@ -2999,7 +2999,7 @@
         <v>34</v>
       </c>
       <c r="C3" s="2" t="n">
-        <v>-14104.225</v>
+        <v>-14123.274</v>
       </c>
     </row>
     <row r="4">
@@ -3010,7 +3010,7 @@
         <v>32</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>5905.441</v>
+        <v>5956.198</v>
       </c>
     </row>
     <row r="5">
@@ -3021,7 +3021,7 @@
         <v>36</v>
       </c>
       <c r="C5" s="2" t="n">
-        <v>1104.568</v>
+        <v>1204.538</v>
       </c>
     </row>
     <row r="6">
@@ -3032,7 +3032,7 @@
         <v>38</v>
       </c>
       <c r="C6" s="2" t="n">
-        <v>4329.42</v>
+        <v>4347.278</v>
       </c>
     </row>
     <row r="7">
@@ -3043,7 +3043,7 @@
         <v>44</v>
       </c>
       <c r="C7" s="2" t="n">
-        <v>6255.995</v>
+        <v>6302.997</v>
       </c>
     </row>
     <row r="8">
@@ -3054,7 +3054,7 @@
         <v>48</v>
       </c>
       <c r="C8" s="2" t="n">
-        <v>-1251.478</v>
+        <v>-1246.266</v>
       </c>
     </row>
     <row r="9">
@@ -3065,7 +3065,7 @@
         <v>56</v>
       </c>
       <c r="C9" s="2" t="n">
-        <v>661.588</v>
+        <v>631.572</v>
       </c>
     </row>
     <row r="10">
@@ -3076,7 +3076,7 @@
         <v>46</v>
       </c>
       <c r="C10" s="2" t="n">
-        <v>1481.145</v>
+        <v>1472.12</v>
       </c>
     </row>
     <row r="11">
@@ -3087,7 +3087,7 @@
         <v>60</v>
       </c>
       <c r="C11" s="2" t="n">
-        <v>-990.668</v>
+        <v>-1001.03</v>
       </c>
     </row>
     <row r="12">
@@ -3098,7 +3098,7 @@
         <v>58</v>
       </c>
       <c r="C12" s="2" t="n">
-        <v>1878.029</v>
+        <v>1879.372</v>
       </c>
     </row>
     <row r="13">
@@ -3109,7 +3109,7 @@
         <v>42</v>
       </c>
       <c r="C13" s="2" t="n">
-        <v>-2697.904</v>
+        <v>-2696.539</v>
       </c>
     </row>
     <row r="14">
@@ -3120,7 +3120,7 @@
         <v>50</v>
       </c>
       <c r="C14" s="2" t="n">
-        <v>-669.754</v>
+        <v>-722.903</v>
       </c>
     </row>
     <row r="15">
@@ -3131,7 +3131,7 @@
         <v>80</v>
       </c>
       <c r="C15" s="2" t="n">
-        <v>-2785.775</v>
+        <v>-2793.309</v>
       </c>
     </row>
     <row r="16">
@@ -3142,7 +3142,7 @@
         <v>68</v>
       </c>
       <c r="C16" s="2" t="n">
-        <v>9419.048</v>
+        <v>9417.832</v>
       </c>
     </row>
     <row r="17">
@@ -3153,7 +3153,7 @@
         <v>78</v>
       </c>
       <c r="C17" s="2" t="n">
-        <v>-698.801</v>
+        <v>-695.757</v>
       </c>
     </row>
     <row r="18">
@@ -3164,7 +3164,7 @@
         <v>66</v>
       </c>
       <c r="C18" s="2" t="n">
-        <v>1305.262</v>
+        <v>1289.308</v>
       </c>
     </row>
     <row r="19">
@@ -3175,7 +3175,7 @@
         <v>64</v>
       </c>
       <c r="C19" s="2" t="n">
-        <v>-1003.137</v>
+        <v>-979.715</v>
       </c>
     </row>
     <row r="20">
@@ -3186,7 +3186,7 @@
         <v>76</v>
       </c>
       <c r="C20" s="2" t="n">
-        <v>-738.207</v>
+        <v>-742.693</v>
       </c>
     </row>
     <row r="21">
@@ -3197,7 +3197,7 @@
         <v>88</v>
       </c>
       <c r="C21" s="2" t="n">
-        <v>-15.633</v>
+        <v>-64.784</v>
       </c>
     </row>
     <row r="22">
@@ -3208,7 +3208,7 @@
         <v>74</v>
       </c>
       <c r="C22" s="2" t="n">
-        <v>-195.373</v>
+        <v>-203.208</v>
       </c>
     </row>
     <row r="23">
@@ -3219,7 +3219,7 @@
         <v>54</v>
       </c>
       <c r="C23" s="2" t="n">
-        <v>-5800.898</v>
+        <v>-5818.718</v>
       </c>
     </row>
     <row r="24">
@@ -3230,7 +3230,7 @@
         <v>70</v>
       </c>
       <c r="C24" s="2" t="n">
-        <v>1046.645</v>
+        <v>1021.028</v>
       </c>
     </row>
     <row r="25">
@@ -3241,7 +3241,7 @@
         <v>82</v>
       </c>
       <c r="C25" s="2" t="n">
-        <v>1834.305</v>
+        <v>1843.613</v>
       </c>
     </row>
     <row r="26">
@@ -3252,7 +3252,7 @@
         <v>92</v>
       </c>
       <c r="C26" s="2" t="n">
-        <v>-614.545</v>
+        <v>-610.542</v>
       </c>
     </row>
     <row r="27">
@@ -3263,7 +3263,7 @@
         <v>84</v>
       </c>
       <c r="C27" s="2" t="n">
-        <v>78.271</v>
+        <v>74.324</v>
       </c>
     </row>
     <row r="28">
@@ -3274,7 +3274,7 @@
         <v>40</v>
       </c>
       <c r="C28" s="2" t="n">
-        <v>-2896.17</v>
+        <v>-2936.188</v>
       </c>
     </row>
     <row r="29">
@@ -3285,7 +3285,7 @@
         <v>86</v>
       </c>
       <c r="C29" s="2" t="n">
-        <v>-2101.823</v>
+        <v>-2105.473</v>
       </c>
     </row>
     <row r="30">
@@ -3296,7 +3296,7 @@
         <v>62</v>
       </c>
       <c r="C30" s="2" t="n">
-        <v>-985.265</v>
+        <v>-1025.562</v>
       </c>
     </row>
     <row r="31">
@@ -3307,7 +3307,7 @@
         <v>30</v>
       </c>
       <c r="C31" s="2" t="n">
-        <v>-1799.116</v>
+        <v>-1814.084</v>
       </c>
     </row>
   </sheetData>
@@ -4059,7 +4059,7 @@
         <v>28</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>-74558.531</v>
+        <v>-73067.452</v>
       </c>
     </row>
     <row r="3">
@@ -4070,7 +4070,7 @@
         <v>36</v>
       </c>
       <c r="C3" s="2" t="n">
-        <v>-12713.317</v>
+        <v>-12783.428</v>
       </c>
     </row>
     <row r="4">
@@ -4081,7 +4081,7 @@
         <v>34</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>-4604.121</v>
+        <v>-4803.282</v>
       </c>
     </row>
     <row r="5">
@@ -4092,7 +4092,7 @@
         <v>32</v>
       </c>
       <c r="C5" s="2" t="n">
-        <v>2287.981</v>
+        <v>2093.5</v>
       </c>
     </row>
     <row r="6">
@@ -4103,7 +4103,7 @@
         <v>52</v>
       </c>
       <c r="C6" s="2" t="n">
-        <v>30765.014</v>
+        <v>30764.009</v>
       </c>
     </row>
     <row r="7">
@@ -4114,7 +4114,7 @@
         <v>38</v>
       </c>
       <c r="C7" s="2" t="n">
-        <v>-1379.559</v>
+        <v>-1515.433</v>
       </c>
     </row>
     <row r="8">
@@ -4125,7 +4125,7 @@
         <v>42</v>
       </c>
       <c r="C8" s="2" t="n">
-        <v>5333.041</v>
+        <v>5316.831</v>
       </c>
     </row>
     <row r="9">
@@ -4136,7 +4136,7 @@
         <v>72</v>
       </c>
       <c r="C9" s="2" t="n">
-        <v>20384.753</v>
+        <v>20384.254</v>
       </c>
     </row>
     <row r="10">
@@ -4147,7 +4147,7 @@
         <v>30</v>
       </c>
       <c r="C10" s="2" t="n">
-        <v>6408.027</v>
+        <v>6403.918</v>
       </c>
     </row>
     <row r="11">
@@ -4158,7 +4158,7 @@
         <v>44</v>
       </c>
       <c r="C11" s="2" t="n">
-        <v>1613.29</v>
+        <v>1583.568</v>
       </c>
     </row>
     <row r="12">
@@ -4169,7 +4169,7 @@
         <v>62</v>
       </c>
       <c r="C12" s="2" t="n">
-        <v>7037.44</v>
+        <v>7036.228</v>
       </c>
     </row>
     <row r="13">
@@ -4180,7 +4180,7 @@
         <v>40</v>
       </c>
       <c r="C13" s="2" t="n">
-        <v>6014.709</v>
+        <v>6003.991</v>
       </c>
     </row>
     <row r="14">
@@ -4191,7 +4191,7 @@
         <v>64</v>
       </c>
       <c r="C14" s="2" t="n">
-        <v>-2949.775</v>
+        <v>-2965.122</v>
       </c>
     </row>
     <row r="15">
@@ -4202,7 +4202,7 @@
         <v>54</v>
       </c>
       <c r="C15" s="2" t="n">
-        <v>-5600.466</v>
+        <v>-5690.251</v>
       </c>
     </row>
     <row r="16">
@@ -4213,7 +4213,7 @@
         <v>60</v>
       </c>
       <c r="C16" s="2" t="n">
-        <v>-2499.225</v>
+        <v>-2619.315</v>
       </c>
     </row>
     <row r="17">
@@ -4224,7 +4224,7 @@
         <v>50</v>
       </c>
       <c r="C17" s="2" t="n">
-        <v>-150.758</v>
+        <v>-172.9</v>
       </c>
     </row>
     <row r="18">
@@ -4235,7 +4235,7 @@
         <v>56</v>
       </c>
       <c r="C18" s="2" t="n">
-        <v>-863.038</v>
+        <v>-887.311</v>
       </c>
     </row>
     <row r="19">
@@ -4246,7 +4246,7 @@
         <v>46</v>
       </c>
       <c r="C19" s="2" t="n">
-        <v>-1368.358</v>
+        <v>-1427.095</v>
       </c>
     </row>
     <row r="20">
@@ -4257,7 +4257,7 @@
         <v>98</v>
       </c>
       <c r="C20" s="2" t="n">
-        <v>3782.806</v>
+        <v>3780.361</v>
       </c>
     </row>
     <row r="21">
@@ -4268,7 +4268,7 @@
         <v>66</v>
       </c>
       <c r="C21" s="2" t="n">
-        <v>2577.66</v>
+        <v>2556.804</v>
       </c>
     </row>
     <row r="22">
@@ -4279,29 +4279,29 @@
         <v>48</v>
       </c>
       <c r="C22" s="2" t="n">
-        <v>-314.964</v>
+        <v>-325.268</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>93</v>
+        <v>101</v>
       </c>
       <c r="B23" t="s">
-        <v>94</v>
+        <v>102</v>
       </c>
       <c r="C23" s="2" t="n">
-        <v>4695.384</v>
+        <v>659.785</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="s">
-        <v>101</v>
+        <v>93</v>
       </c>
       <c r="B24" t="s">
-        <v>102</v>
+        <v>94</v>
       </c>
       <c r="C24" s="2" t="n">
-        <v>666.766</v>
+        <v>4690.68</v>
       </c>
     </row>
     <row r="25">
@@ -4312,7 +4312,7 @@
         <v>70</v>
       </c>
       <c r="C25" s="2" t="n">
-        <v>1474.973</v>
+        <v>1445.439</v>
       </c>
     </row>
     <row r="26">
@@ -4323,7 +4323,7 @@
         <v>78</v>
       </c>
       <c r="C26" s="2" t="n">
-        <v>571.952</v>
+        <v>561.358</v>
       </c>
     </row>
     <row r="27">
@@ -4334,29 +4334,29 @@
         <v>74</v>
       </c>
       <c r="C27" s="2" t="n">
-        <v>-1860.016</v>
+        <v>-1926.339</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="s">
-        <v>75</v>
+        <v>87</v>
       </c>
       <c r="B28" t="s">
-        <v>76</v>
+        <v>88</v>
       </c>
       <c r="C28" s="2" t="n">
-        <v>-442.846</v>
+        <v>-1471.035</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="s">
-        <v>87</v>
+        <v>75</v>
       </c>
       <c r="B29" t="s">
-        <v>88</v>
+        <v>76</v>
       </c>
       <c r="C29" s="2" t="n">
-        <v>-1411.058</v>
+        <v>-449.153</v>
       </c>
     </row>
     <row r="30">
@@ -4367,7 +4367,7 @@
         <v>84</v>
       </c>
       <c r="C30" s="2" t="n">
-        <v>-230.671</v>
+        <v>-240.453</v>
       </c>
     </row>
     <row r="31">
@@ -4378,7 +4378,7 @@
         <v>82</v>
       </c>
       <c r="C31" s="2" t="n">
-        <v>-563.393</v>
+        <v>-568.07</v>
       </c>
     </row>
   </sheetData>
@@ -4416,7 +4416,7 @@
         <v>28</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>-205919.279</v>
+        <v>-205918.171</v>
       </c>
     </row>
     <row r="3">
@@ -4427,7 +4427,7 @@
         <v>30</v>
       </c>
       <c r="C3" s="2" t="n">
-        <v>93952.215</v>
+        <v>93952.14</v>
       </c>
     </row>
     <row r="4">
@@ -4460,7 +4460,7 @@
         <v>34</v>
       </c>
       <c r="C6" s="2" t="n">
-        <v>-3532.775</v>
+        <v>-3533.396</v>
       </c>
     </row>
     <row r="7">
@@ -4493,7 +4493,7 @@
         <v>32</v>
       </c>
       <c r="C9" s="2" t="n">
-        <v>-3573.227</v>
+        <v>-3573.008</v>
       </c>
     </row>
     <row r="10">
@@ -4526,7 +4526,7 @@
         <v>54</v>
       </c>
       <c r="C12" s="2" t="n">
-        <v>-2736.215</v>
+        <v>-2736.273</v>
       </c>
     </row>
     <row r="13">
@@ -4548,7 +4548,7 @@
         <v>66</v>
       </c>
       <c r="C14" s="2" t="n">
-        <v>4926.08</v>
+        <v>5007.723</v>
       </c>
     </row>
     <row r="15">
@@ -4592,7 +4592,7 @@
         <v>64</v>
       </c>
       <c r="C18" s="2" t="n">
-        <v>-1822.405</v>
+        <v>-1822.548</v>
       </c>
     </row>
     <row r="19">
@@ -4614,7 +4614,7 @@
         <v>48</v>
       </c>
       <c r="C20" s="2" t="n">
-        <v>-664.269</v>
+        <v>-664.05</v>
       </c>
     </row>
     <row r="21">
@@ -4702,7 +4702,7 @@
         <v>70</v>
       </c>
       <c r="C28" s="2" t="n">
-        <v>-1772.467</v>
+        <v>-1772.589</v>
       </c>
     </row>
     <row r="29">
@@ -4713,7 +4713,7 @@
         <v>86</v>
       </c>
       <c r="C29" s="2" t="n">
-        <v>-191.386</v>
+        <v>-259.719</v>
       </c>
     </row>
     <row r="30">

</xml_diff>